<commit_message>
Improve RAG retrieval and knowledge workflows
</commit_message>
<xml_diff>
--- a/docs/knowledge-base/tickets.xlsx
+++ b/docs/knowledge-base/tickets.xlsx
@@ -10,7 +10,10 @@
     <sheet name="tickets" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="deploy_history" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tickets'!$A$1:$M$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'deploy_history'!$A$1:$E$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +29,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017324D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +59,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,170 +432,830 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ticket_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>service_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>incident_type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>root_cause</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>excluded_hypotheses</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>decision_record</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>resolution</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>evidence</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>approval_record</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>rollback_condition</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="66" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>INC-REDIS-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>order-service</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>redis_maxclients</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Checkout 5xx peaked at 12.8% for 18 minutes</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Redis maxclients exhausted by retry storm</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Redis CPU saturation; packet loss; single slow command</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed after temporal ordering, mechanism evidence, and canary reversal</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Reduced retry amplification and raised maxclients after approval</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>connected_clients=9940 maxclients=10000 blocked_clients=37</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>CR-REDIS-2026-071 approved by Incident Commander and Redis Owner</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Checkout 5xx or replication lag increases during canary</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Commerce Platform SRE</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="66" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>INC-REDIS-009</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>order-service</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>redis_maxclients</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Promotion lookup retry loop exhausted Redis client slots</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>促销查询重试超时 delayed order confirmation</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>促销查询重试循环 exhausted Redis client slots and maxclients headroom</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Network loss; Redis host CPU; command latency</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by release ownership and client-pressure reversal</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Reduced retry burst and capped idle Redis pool after approval</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Loki redis timeout Prometheus 5xx connected_clients near maxclients</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Order Platform and Redis Owner approved 10% canary</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Client churn, blocked clients, or 5xx increases</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Order Platform</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="66" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>INC-MYSQL-014</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>payment-service</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>mysql_slow_query</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Payment P95 reached 5.2 seconds and timeout rate reached 9.6%</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Slow SQL held MySQL connections and caused pool waiting</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Database host CPU; network latency; permanent connection leak</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by digest, EXPLAIN, hold time, and canary reversal</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Captured digest, added index after approval, observed P95 recovery</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>slow_queries=18 active_connections=188/200 pool_waiting=6</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>CR-MYSQL-2026-044 approved by Payments Owner and DBA</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Lock wait, replica lag, or payment errors increase</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Payments Reliability</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="66" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>INC-MYSQL-021</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>payment-service</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>mysql_pool_waiting</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Checkout requests queued while idempotency prevented duplicate charges</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Checkout report query caused MySQL pool_waiting after release rc3</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Connection leak; packet loss; storage saturation</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed after feature disable cleared pool waiting</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Disabled report flag, reviewed EXPLAIN, then added covering index</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>deploy rc3 slow query digest payment_report_join_v3 pool_waiting=6</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Feature canary approved before the later DBA index change</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Payment errors exceed 2% or replica lag exceeds 10 seconds</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Payments Reliability</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>INC-NET-027</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>gateway-service</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>network_timeout</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Cross-zone connect latency caused intermittent upstream 504 responses</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>SNAT port pressure amplified by short-lived retry connections</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>DNS resolution; TLS expiry; application first-byte latency</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by network-stage decomposition and connection canary</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Reduced retry concurrency and shifted a 10% canary after approval</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>connect latency retransmits conntrack and SNAT utilization aligned</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Network Platform approved route canary CR-NET-2026-027</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Packet loss, cross-zone cost, or downstream connections increase</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Network Platform</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>INC-TLS-011</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>public-api</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>tls_certificate_expiry</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>A subset of older clients failed TLS handshake at one ingress</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>One ingress retained an expired certificate binding</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Client clock skew; DNS mismatch; unsupported cipher</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by node-specific certificate serial and binding comparison</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Applied dual-certificate canary and reloaded the ingress after approval</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>SNI serial notAfter and ingress binding differed on one node</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Security Platform and API Owner approved CR-TLS-2026-011</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Handshake failures or legacy-client failures increase</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Security Platform</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>INC-DNS-019</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>catalog-service</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>dns_resolution_failure</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Pods intermittently returned no such host for an internal dependency</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>CoreDNS upstream timeout combined with stale negative cache</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Authoritative record error; service endpoint failure; TCP routing</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by resolver comparison and CoreDNS upstream timing</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Canaried an upstream resolver change after preserving DNS evidence</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>SERVFAIL coredns latency and Pod resolver comparison</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Kubernetes Platform approved CR-DNS-2026-019</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>NXDOMAIN, wrong-address answers, or traffic skew increases</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Kubernetes Platform</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>INC-THREAD-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>inventory-service</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>thread_pool_exhaustion</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Request queue growth pushed inventory P99 above eight seconds</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Worker threads blocked on a slow downstream API</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>CPU saturation; database pool leak; garbage collection</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by thread stacks and downstream span duration</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Reduced downstream concurrency and enabled approved backpressure canary</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>thread dumps queue depth rejected tasks and downstream trace spans</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Owner approved CR-THREAD-2026-008</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Rejected tasks, downstream connections, or error rate increases</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Platform</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="66" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>INC-MQ-023</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>fulfillment-consumer</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>message_queue_backlog</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Oldest fulfillment event age reached 26 minutes</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>A poison message triggered repeated consumer retries on one partition</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Producer surge; broker disk saturation; broad consumer shortage</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by single-message and single-partition concentration</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Quarantined the message and replayed at a capped rate after approval</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>single partition lag repeated message key and downstream validation error</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Messaging Platform and Fulfillment Owner approved replay</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate processing, rebalance, or downstream errors increase</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Messaging Platform</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>INC-K8S-031</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>recommendation-worker</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>kubernetes_scheduling_failure</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>New worker replicas remained Pending and reduced batch throughput</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Resource requests and zone affinity left no eligible node</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Container image failure; application crash; PVC outage</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by scheduler events and eligible-node calculation</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted one canary workload constraint after platform approval</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>FailedScheduling events requests allocatable capacity and affinity</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Kubernetes Platform approved CR-K8S-2026-031</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Wrong-zone placement, resource contention, or instability appears</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Kubernetes Platform</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>INC-MYSQL-LOCK-017</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>billing-service</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>mysql_lock_wait</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Invoice updates queued and API timeout rate reached 6.4%</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>A long batch transaction blocked the online update path</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Slow storage; connection leak; database CPU saturation</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by lock graph, transaction age, and recovery after rollback</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Paused the batch and rolled back the blocker after DBA approval</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>performance_schema lock graph transaction age digest and pool waiting</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>DBA and Billing Owner approved CR-LOCK-2026-017</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Replica lag, rollback volume, or data mismatch increases</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Database Platform</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -590,143 +1268,151 @@
   </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>service_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>deployed_at</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>change_summary</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>risk_hint</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="66" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>payment-service</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>payment-api-2026.07.06-rc3</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>2026-07-06T09:42:00Z</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Changed checkout order query path and ORM eager loading</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Correlates with slow query and pool_waiting=6</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="66" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>payment-service</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>payment-api-2026.07.06-rc4</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>2026-07-06T10:32:00Z</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Disabled checkout report feature flag and prepared index change</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Remediation after approval; not an automatically executed Agent action</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="66" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>order-service</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>order-api-2026.07.06-rc1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>2026-07-06T09:10:00Z</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Raised Redis retry count in promotion lookup path</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Can amplify Redis maxclients pressure</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="66" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>order-service</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>order-api-2026.07.06-rc2</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>2026-07-06T10:28:00Z</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Reduced Redis retry count and idle pool retention</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Remediation after approval for maxclients pressure</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>